<commit_message>
Improve registration tracking, public URLs, and award validation.
Use REG reference numbers, keep tracking photos on-page, and add public /track routing for local and hosted testing.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/tocca_admin/uploads/tocca_import_template.xlsx
+++ b/tocca_admin/uploads/tocca_import_template.xlsx
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="113">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="138">
   <si>
     <t>TOCCA — Excel import guide (read this first)</t>
   </si>
@@ -27,10 +27,10 @@
     <t>WHAT THIS FILE IS FOR</t>
   </si>
   <si>
-    <t>Use this workbook to load Categories, Name of Awards, Establishment Types, and Establishments into the active event.</t>
-  </si>
-  <si>
-    <t>Fill in the four data sheets, then upload the file from Admin → System Utilities → Import Data.</t>
+    <t>Use this workbook to load Categories, Awards, Establishment Types, and Establishments into the active event.</t>
+  </si>
+  <si>
+    <t>Fill in the four data sheets, then upload from Admin → System Utilities → Import Data.</t>
   </si>
   <si>
     <t>BEFORE YOU START</t>
@@ -45,12 +45,33 @@
     <t>• Row 1 on each data sheet is a hint row. Row 2 is the column header row. Your data starts on row 3.</t>
   </si>
   <si>
-    <t>• The sample rows below the headers WILL be imported — edit them to your real event data before uploading.</t>
+    <t>• The sample rows below the headers WILL be imported — replace them with your real event data before uploading.</t>
   </si>
   <si>
     <t>• Fill sheets in this order: Categories → Awards → Establishment Types → Establishments.</t>
   </si>
   <si>
+    <t>IMPORTANT — Linking awards to establishment types</t>
+  </si>
+  <si>
+    <t>• The Establishment Types sheet is how awards get linked to business types automatically.</t>
+  </si>
+  <si>
+    <t>• If you import Categories + Awards only (and leave Establishment Types empty/missing), new awards will NOT</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  appear under any type on the registration form until an admin links them under File Maintenance → Establishment Types.</t>
+  </si>
+  <si>
+    <t>• Always fill award_keys on the Establishment Types sheet so applicants see the right awards after import.</t>
+  </si>
+  <si>
+    <t>• On the public registration form, applicants can select ONE OR MORE establishment types (checkboxes).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  Awards shown are the combined list for all types they selected.</t>
+  </si>
+  <si>
     <t>QUICK GLOSSARY (plain English)</t>
   </si>
   <si>
@@ -84,7 +105,7 @@
     <t xml:space="preserve">  A short code YOU create for each award — the system does not generate this for you.</t>
   </si>
   <si>
-    <t xml:space="preserve">  Examples: F1, F2, S1, FE1, FU1</t>
+    <t xml:space="preserve">  Examples: F1, F2, S1, FE1, R1</t>
   </si>
   <si>
     <t xml:space="preserve">  Rules:</t>
@@ -111,25 +132,19 @@
     <t>choice_type</t>
   </si>
   <si>
-    <t xml:space="preserve">  How voters answer this award during e-voting.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">  • 1 = Options — voter picks from a list of establishments (use this for normal nominee awards)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">  • 0 = Freeform — voter types their own text answer (rare; use only for open-ended questions)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">  For TOCCA establishment awards, almost always use 1.</t>
+    <t xml:space="preserve">  Always use 1 (Options). Voters pick from linked establishments.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  Freeform (0) is not used on the voting page and is ignored on import.</t>
   </si>
   <si>
     <t>type_name (Establishment Types sheet)</t>
   </si>
   <si>
-    <t xml:space="preserve">  The kind of business (e.g. Restaurant, Salon, Grocery).</t>
-  </si>
-  <si>
-    <t xml:space="preserve">  This appears on the nomination form as “Establishment Type”.</t>
+    <t xml:space="preserve">  The kind of business (e.g. Restaurant, Café, Hair Salon).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  This appears on the registration form as “Establishment Type” (multi-select checkboxes).</t>
   </si>
   <si>
     <t>award_keys (Establishment Types sheet)</t>
@@ -141,7 +156,10 @@
     <t xml:space="preserve">  Copy the award_key values from the Awards sheet, separated by commas.</t>
   </si>
   <si>
-    <t xml:space="preserve">  Example: F1, FU1  means this type can participate in awards F1 and FU1.</t>
+    <t xml:space="preserve">  Example: F1, F2  means this type can participate in awards F1 and F2.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  The same award_key may appear under more than one type (e.g. Best Burger for Restaurant and Fast Food).</t>
   </si>
   <si>
     <t>establishment_type (Establishments sheet)</t>
@@ -150,6 +168,9 @@
     <t xml:space="preserve">  Must match a type_name from the Establishment Types sheet exactly.</t>
   </si>
   <si>
+    <t xml:space="preserve">  One type per row for bulk import. To assign additional types later, edit the establishment in Admin.</t>
+  </si>
+  <si>
     <t>award_key (Establishments sheet)</t>
   </si>
   <si>
@@ -174,7 +195,7 @@
     <t xml:space="preserve">   award_key | category_name | award_name | choice_type</t>
   </si>
   <si>
-    <t>3) Establishment Types — one row per business type</t>
+    <t>3) Establishment Types — one row per business type (REQUIRED to auto-link awards)</t>
   </si>
   <si>
     <t xml:space="preserve">   type_name | award_keys | status</t>
@@ -195,6 +216,9 @@
     <t>• Using award_name instead of award_key on Establishment Types / Establishments</t>
   </si>
   <si>
+    <t>• Importing awards without filling Establishment Types — then wondering why types have no awards</t>
+  </si>
+  <si>
     <t>• Listing an award under a type that was not assigned in Establishment Types</t>
   </si>
   <si>
@@ -228,9 +252,6 @@
     <t>Feelings</t>
   </si>
   <si>
-    <t>Fun</t>
-  </si>
-  <si>
     <t>Short unique code YOU invent (e.g. F1). Copy to other sheets. Do not use spaces.</t>
   </si>
   <si>
@@ -240,43 +261,73 @@
     <t>Full award title voters will see (e.g. Best Chicken Barbecue).</t>
   </si>
   <si>
-    <t>1 = Options (pick establishments). 0 = Freeform (typed answer). Use 1 for normal awards.</t>
+    <t>Always 1 = Options (pick establishments). Freeform is not used for voting.</t>
   </si>
   <si>
     <t>F1</t>
   </si>
   <si>
+    <t>Best Burger</t>
+  </si>
+  <si>
+    <t>F2</t>
+  </si>
+  <si>
     <t>Best Chicken Barbecue</t>
   </si>
   <si>
+    <t>F3</t>
+  </si>
+  <si>
+    <t>Best Pancit</t>
+  </si>
+  <si>
     <t>S1</t>
   </si>
   <si>
+    <t>Best Café</t>
+  </si>
+  <si>
+    <t>S2</t>
+  </si>
+  <si>
     <t>Best Hair Salon</t>
   </si>
   <si>
+    <t>S3</t>
+  </si>
+  <si>
+    <t>Best Catering Services</t>
+  </si>
+  <si>
     <t>R1</t>
   </si>
   <si>
     <t>Best Grocery Shop</t>
   </si>
   <si>
+    <t>R2</t>
+  </si>
+  <si>
+    <t>Best Meat Shop</t>
+  </si>
+  <si>
     <t>FE1</t>
   </si>
   <si>
     <t>Best Date Place</t>
   </si>
   <si>
-    <t>FU1</t>
-  </si>
-  <si>
-    <t>Best Karaoke Bar</t>
-  </si>
-  <si>
-    <t>Business type name (e.g. Restaurant). Shown on the nomination form.</t>
-  </si>
-  <si>
-    <t>award_key codes from Awards sheet, comma-separated (e.g. F1, FU1).</t>
+    <t>FE2</t>
+  </si>
+  <si>
+    <t>Best Hairstylist</t>
+  </si>
+  <si>
+    <t>Business type name (e.g. Restaurant). Shown as checkboxes on the registration form.</t>
+  </si>
+  <si>
+    <t>award_key codes from Awards sheet, comma-separated (e.g. F1, F2). Links awards to this type.</t>
   </si>
   <si>
     <t>1 = Active. 0 = Inactive.</t>
@@ -288,22 +339,46 @@
     <t>award_keys</t>
   </si>
   <si>
+    <t>Café</t>
+  </si>
+  <si>
+    <t>S1, FE1</t>
+  </si>
+  <si>
     <t>Restaurant</t>
   </si>
   <si>
-    <t>F1, FU1</t>
-  </si>
-  <si>
-    <t>Salon</t>
-  </si>
-  <si>
-    <t>Grocery</t>
-  </si>
-  <si>
-    <t>Date Spot</t>
-  </si>
-  <si>
-    <t>Karaoke Bar</t>
+    <t>F1, F2, F3, S3, FE1</t>
+  </si>
+  <si>
+    <t>Fast Food Chain</t>
+  </si>
+  <si>
+    <t>F1, F2</t>
+  </si>
+  <si>
+    <t>Bakery / Pastry Shop</t>
+  </si>
+  <si>
+    <t>Carinderia / Eatery</t>
+  </si>
+  <si>
+    <t>F2, F3</t>
+  </si>
+  <si>
+    <t>Catering Service</t>
+  </si>
+  <si>
+    <t>Grocery / Mini Mart</t>
+  </si>
+  <si>
+    <t>Meat Shop</t>
+  </si>
+  <si>
+    <t>Hair Salon</t>
+  </si>
+  <si>
+    <t>S2, FE2</t>
   </si>
   <si>
     <t>Official business / establishment name.</t>
@@ -315,7 +390,7 @@
     <t>1 = Active nominee. 0 = Inactive.</t>
   </si>
   <si>
-    <t>Must match type_name on Establishment Types sheet.</t>
+    <t>Must match type_name on Establishment Types sheet (one type per import row).</t>
   </si>
   <si>
     <t>award_key from Awards sheet. One award per row — duplicate the row for multiple awards.</t>
@@ -342,10 +417,10 @@
     <t>angels.burger@test.local</t>
   </si>
   <si>
-    <t>Dongski Barbershop</t>
-  </si>
-  <si>
-    <t>dongski@test.local</t>
+    <t>Bean &amp; Brew Café</t>
+  </si>
+  <si>
+    <t>beanbrew@test.local</t>
   </si>
   <si>
     <t>Ormoc Centrum</t>
@@ -354,10 +429,10 @@
     <t>ormoc.centrum@test.local</t>
   </si>
   <si>
-    <t>Rosario's Flower Shop</t>
-  </si>
-  <si>
-    <t>rosarios.flowers@test.local</t>
+    <t>Style Cut Salon</t>
+  </si>
+  <si>
+    <t>stylecut@test.local</t>
   </si>
 </sst>
 </file>
@@ -717,7 +792,7 @@
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
   </sheetPr>
-  <dimension ref="A1:E82"/>
+  <dimension ref="A1:E91"/>
   <sheetFormatPr defaultRowHeight="14.4" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col min="1" max="1" width="28" customWidth="true" style="0"/>
@@ -782,38 +857,38 @@
         <v>10</v>
       </c>
     </row>
+    <row r="15" spans="1:5">
+      <c r="A15" t="s">
+        <v>11</v>
+      </c>
+    </row>
     <row r="16" spans="1:5">
       <c r="A16" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
     </row>
     <row r="17" spans="1:5">
       <c r="A17" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
     </row>
     <row r="18" spans="1:5">
       <c r="A18" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
     </row>
     <row r="19" spans="1:5">
       <c r="A19" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
     </row>
     <row r="20" spans="1:5">
       <c r="A20" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
     </row>
     <row r="22" spans="1:5">
       <c r="A22" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="23" spans="1:5">
-      <c r="A23" t="s">
         <v>17</v>
       </c>
     </row>
@@ -822,23 +897,23 @@
         <v>18</v>
       </c>
     </row>
+    <row r="25" spans="1:5">
+      <c r="A25" t="s">
+        <v>19</v>
+      </c>
+    </row>
     <row r="26" spans="1:5">
       <c r="A26" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
     </row>
     <row r="27" spans="1:5">
       <c r="A27" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
     </row>
     <row r="28" spans="1:5">
       <c r="A28" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="29" spans="1:5">
-      <c r="A29" t="s">
         <v>22</v>
       </c>
     </row>
@@ -857,8 +932,8 @@
         <v>25</v>
       </c>
     </row>
-    <row r="33" spans="1:5">
-      <c r="A33" t="s">
+    <row r="34" spans="1:5">
+      <c r="A34" t="s">
         <v>26</v>
       </c>
     </row>
@@ -872,38 +947,38 @@
         <v>28</v>
       </c>
     </row>
+    <row r="37" spans="1:5">
+      <c r="A37" t="s">
+        <v>29</v>
+      </c>
+    </row>
     <row r="38" spans="1:5">
       <c r="A38" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
     </row>
     <row r="39" spans="1:5">
       <c r="A39" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
     </row>
     <row r="40" spans="1:5">
       <c r="A40" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
     </row>
     <row r="41" spans="1:5">
       <c r="A41" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="42" spans="1:5">
-      <c r="A42" t="s">
         <v>33</v>
+      </c>
+    </row>
+    <row r="43" spans="1:5">
+      <c r="A43" t="s">
+        <v>34</v>
       </c>
     </row>
     <row r="44" spans="1:5">
       <c r="A44" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="45" spans="1:5">
-      <c r="A45" t="s">
         <v>35</v>
       </c>
     </row>
@@ -912,13 +987,13 @@
         <v>36</v>
       </c>
     </row>
+    <row r="47" spans="1:5">
+      <c r="A47" t="s">
+        <v>37</v>
+      </c>
+    </row>
     <row r="48" spans="1:5">
       <c r="A48" t="s">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="49" spans="1:5">
-      <c r="A49" t="s">
         <v>38</v>
       </c>
     </row>
@@ -932,8 +1007,8 @@
         <v>40</v>
       </c>
     </row>
-    <row r="53" spans="1:5">
-      <c r="A53" t="s">
+    <row r="52" spans="1:5">
+      <c r="A52" t="s">
         <v>41</v>
       </c>
     </row>
@@ -942,88 +1017,88 @@
         <v>42</v>
       </c>
     </row>
+    <row r="55" spans="1:5">
+      <c r="A55" t="s">
+        <v>43</v>
+      </c>
+    </row>
     <row r="56" spans="1:5">
       <c r="A56" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
     </row>
     <row r="57" spans="1:5">
       <c r="A57" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
     </row>
     <row r="58" spans="1:5">
       <c r="A58" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
     </row>
     <row r="60" spans="1:5">
       <c r="A60" t="s">
-        <v>46</v>
+        <v>47</v>
+      </c>
+    </row>
+    <row r="61" spans="1:5">
+      <c r="A61" t="s">
+        <v>48</v>
       </c>
     </row>
     <row r="62" spans="1:5">
       <c r="A62" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="63" spans="1:5">
-      <c r="A63" t="s">
-        <v>48</v>
+        <v>49</v>
+      </c>
+    </row>
+    <row r="64" spans="1:5">
+      <c r="A64" t="s">
+        <v>50</v>
       </c>
     </row>
     <row r="65" spans="1:5">
       <c r="A65" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
     </row>
     <row r="66" spans="1:5">
       <c r="A66" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
     </row>
     <row r="68" spans="1:5">
       <c r="A68" t="s">
-        <v>51</v>
-      </c>
-    </row>
-    <row r="69" spans="1:5">
-      <c r="A69" t="s">
-        <v>52</v>
+        <v>53</v>
+      </c>
+    </row>
+    <row r="70" spans="1:5">
+      <c r="A70" t="s">
+        <v>54</v>
       </c>
     </row>
     <row r="71" spans="1:5">
       <c r="A71" t="s">
-        <v>53</v>
-      </c>
-    </row>
-    <row r="72" spans="1:5">
-      <c r="A72" t="s">
-        <v>54</v>
+        <v>55</v>
+      </c>
+    </row>
+    <row r="73" spans="1:5">
+      <c r="A73" t="s">
+        <v>56</v>
       </c>
     </row>
     <row r="74" spans="1:5">
       <c r="A74" t="s">
-        <v>55</v>
-      </c>
-    </row>
-    <row r="75" spans="1:5">
-      <c r="A75" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
     </row>
     <row r="76" spans="1:5">
       <c r="A76" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
     </row>
     <row r="77" spans="1:5">
       <c r="A77" t="s">
-        <v>58</v>
-      </c>
-    </row>
-    <row r="78" spans="1:5">
-      <c r="A78" t="s">
         <v>59</v>
       </c>
     </row>
@@ -1032,14 +1107,54 @@
         <v>60</v>
       </c>
     </row>
-    <row r="81" spans="1:5">
-      <c r="A81" t="s">
+    <row r="80" spans="1:5">
+      <c r="A80" t="s">
         <v>61</v>
       </c>
     </row>
     <row r="82" spans="1:5">
       <c r="A82" t="s">
         <v>62</v>
+      </c>
+    </row>
+    <row r="83" spans="1:5">
+      <c r="A83" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="84" spans="1:5">
+      <c r="A84" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="85" spans="1:5">
+      <c r="A85" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="86" spans="1:5">
+      <c r="A86" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="87" spans="1:5">
+      <c r="A87" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="88" spans="1:5">
+      <c r="A88" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="90" spans="1:5">
+      <c r="A90" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="91" spans="1:5">
+      <c r="A91" t="s">
+        <v>70</v>
       </c>
     </row>
   </sheetData>
@@ -1054,7 +1169,7 @@
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
   </sheetPr>
-  <dimension ref="A1:Z7"/>
+  <dimension ref="A1:Z6"/>
   <sheetFormatPr defaultRowHeight="14.4" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col min="1" max="1" width="28" customWidth="true" style="0"/>
@@ -1066,10 +1181,10 @@
   <sheetData>
     <row r="1" spans="1:26">
       <c r="A1" s="2" t="s">
-        <v>63</v>
+        <v>71</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>64</v>
+        <v>72</v>
       </c>
       <c r="C1" s="2"/>
       <c r="D1" s="2"/>
@@ -1098,10 +1213,10 @@
     </row>
     <row r="2" spans="1:26">
       <c r="A2" s="1" t="s">
-        <v>16</v>
+        <v>23</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>11</v>
+        <v>18</v>
       </c>
       <c r="C2" s="1"/>
       <c r="D2" s="1"/>
@@ -1130,7 +1245,7 @@
     </row>
     <row r="3" spans="1:26">
       <c r="A3" t="s">
-        <v>65</v>
+        <v>73</v>
       </c>
       <c r="B3">
         <v>1</v>
@@ -1138,7 +1253,7 @@
     </row>
     <row r="4" spans="1:26">
       <c r="A4" t="s">
-        <v>66</v>
+        <v>74</v>
       </c>
       <c r="B4">
         <v>1</v>
@@ -1146,7 +1261,7 @@
     </row>
     <row r="5" spans="1:26">
       <c r="A5" t="s">
-        <v>67</v>
+        <v>75</v>
       </c>
       <c r="B5">
         <v>1</v>
@@ -1154,17 +1269,9 @@
     </row>
     <row r="6" spans="1:26">
       <c r="A6" t="s">
-        <v>68</v>
+        <v>76</v>
       </c>
       <c r="B6">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="7" spans="1:26">
-      <c r="A7" t="s">
-        <v>69</v>
-      </c>
-      <c r="B7">
         <v>1</v>
       </c>
     </row>
@@ -1180,7 +1287,7 @@
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
   </sheetPr>
-  <dimension ref="A1:Z7"/>
+  <dimension ref="A1:Z12"/>
   <sheetFormatPr defaultRowHeight="14.4" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col min="1" max="1" width="28" customWidth="true" style="0"/>
@@ -1192,16 +1299,16 @@
   <sheetData>
     <row r="1" spans="1:26">
       <c r="A1" s="2" t="s">
-        <v>70</v>
+        <v>77</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>71</v>
+        <v>78</v>
       </c>
       <c r="C1" s="2" t="s">
-        <v>72</v>
+        <v>79</v>
       </c>
       <c r="D1" s="2" t="s">
-        <v>73</v>
+        <v>80</v>
       </c>
       <c r="E1" s="2"/>
       <c r="F1" s="2"/>
@@ -1228,16 +1335,16 @@
     </row>
     <row r="2" spans="1:26">
       <c r="A2" s="1" t="s">
-        <v>19</v>
+        <v>26</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>16</v>
+        <v>23</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>27</v>
+        <v>34</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>29</v>
+        <v>36</v>
       </c>
       <c r="E2" s="1"/>
       <c r="F2" s="1"/>
@@ -1264,13 +1371,13 @@
     </row>
     <row r="3" spans="1:26">
       <c r="A3" t="s">
-        <v>74</v>
+        <v>81</v>
       </c>
       <c r="B3" t="s">
-        <v>65</v>
+        <v>73</v>
       </c>
       <c r="C3" t="s">
-        <v>75</v>
+        <v>82</v>
       </c>
       <c r="D3">
         <v>1</v>
@@ -1278,13 +1385,13 @@
     </row>
     <row r="4" spans="1:26">
       <c r="A4" t="s">
-        <v>76</v>
+        <v>83</v>
       </c>
       <c r="B4" t="s">
-        <v>66</v>
+        <v>73</v>
       </c>
       <c r="C4" t="s">
-        <v>77</v>
+        <v>84</v>
       </c>
       <c r="D4">
         <v>1</v>
@@ -1292,13 +1399,13 @@
     </row>
     <row r="5" spans="1:26">
       <c r="A5" t="s">
-        <v>78</v>
+        <v>85</v>
       </c>
       <c r="B5" t="s">
-        <v>67</v>
+        <v>73</v>
       </c>
       <c r="C5" t="s">
-        <v>79</v>
+        <v>86</v>
       </c>
       <c r="D5">
         <v>1</v>
@@ -1306,13 +1413,13 @@
     </row>
     <row r="6" spans="1:26">
       <c r="A6" t="s">
-        <v>80</v>
+        <v>87</v>
       </c>
       <c r="B6" t="s">
-        <v>68</v>
+        <v>74</v>
       </c>
       <c r="C6" t="s">
-        <v>81</v>
+        <v>88</v>
       </c>
       <c r="D6">
         <v>1</v>
@@ -1320,15 +1427,85 @@
     </row>
     <row r="7" spans="1:26">
       <c r="A7" t="s">
-        <v>82</v>
+        <v>89</v>
       </c>
       <c r="B7" t="s">
-        <v>69</v>
+        <v>74</v>
       </c>
       <c r="C7" t="s">
-        <v>83</v>
+        <v>90</v>
       </c>
       <c r="D7">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="8" spans="1:26">
+      <c r="A8" t="s">
+        <v>91</v>
+      </c>
+      <c r="B8" t="s">
+        <v>74</v>
+      </c>
+      <c r="C8" t="s">
+        <v>92</v>
+      </c>
+      <c r="D8">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="9" spans="1:26">
+      <c r="A9" t="s">
+        <v>93</v>
+      </c>
+      <c r="B9" t="s">
+        <v>75</v>
+      </c>
+      <c r="C9" t="s">
+        <v>94</v>
+      </c>
+      <c r="D9">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="10" spans="1:26">
+      <c r="A10" t="s">
+        <v>95</v>
+      </c>
+      <c r="B10" t="s">
+        <v>75</v>
+      </c>
+      <c r="C10" t="s">
+        <v>96</v>
+      </c>
+      <c r="D10">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="11" spans="1:26">
+      <c r="A11" t="s">
+        <v>97</v>
+      </c>
+      <c r="B11" t="s">
+        <v>76</v>
+      </c>
+      <c r="C11" t="s">
+        <v>98</v>
+      </c>
+      <c r="D11">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="12" spans="1:26">
+      <c r="A12" t="s">
+        <v>99</v>
+      </c>
+      <c r="B12" t="s">
+        <v>76</v>
+      </c>
+      <c r="C12" t="s">
+        <v>100</v>
+      </c>
+      <c r="D12">
         <v>1</v>
       </c>
     </row>
@@ -1344,7 +1521,7 @@
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
   </sheetPr>
-  <dimension ref="A1:Z7"/>
+  <dimension ref="A1:Z11"/>
   <sheetFormatPr defaultRowHeight="14.4" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col min="1" max="1" width="28" customWidth="true" style="0"/>
@@ -1356,13 +1533,13 @@
   <sheetData>
     <row r="1" spans="1:26">
       <c r="A1" s="2" t="s">
-        <v>84</v>
+        <v>101</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>85</v>
+        <v>102</v>
       </c>
       <c r="C1" s="2" t="s">
-        <v>86</v>
+        <v>103</v>
       </c>
       <c r="D1" s="2"/>
       <c r="E1" s="2"/>
@@ -1390,13 +1567,13 @@
     </row>
     <row r="2" spans="1:26">
       <c r="A2" s="1" t="s">
-        <v>87</v>
+        <v>104</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>88</v>
+        <v>105</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>11</v>
+        <v>18</v>
       </c>
       <c r="D2" s="1"/>
       <c r="E2" s="1"/>
@@ -1424,10 +1601,10 @@
     </row>
     <row r="3" spans="1:26">
       <c r="A3" t="s">
-        <v>89</v>
+        <v>106</v>
       </c>
       <c r="B3" t="s">
-        <v>90</v>
+        <v>107</v>
       </c>
       <c r="C3">
         <v>1</v>
@@ -1435,10 +1612,10 @@
     </row>
     <row r="4" spans="1:26">
       <c r="A4" t="s">
-        <v>91</v>
+        <v>108</v>
       </c>
       <c r="B4" t="s">
-        <v>76</v>
+        <v>109</v>
       </c>
       <c r="C4">
         <v>1</v>
@@ -1446,10 +1623,10 @@
     </row>
     <row r="5" spans="1:26">
       <c r="A5" t="s">
-        <v>92</v>
+        <v>110</v>
       </c>
       <c r="B5" t="s">
-        <v>78</v>
+        <v>111</v>
       </c>
       <c r="C5">
         <v>1</v>
@@ -1457,10 +1634,10 @@
     </row>
     <row r="6" spans="1:26">
       <c r="A6" t="s">
-        <v>93</v>
+        <v>112</v>
       </c>
       <c r="B6" t="s">
-        <v>80</v>
+        <v>87</v>
       </c>
       <c r="C6">
         <v>1</v>
@@ -1468,12 +1645,56 @@
     </row>
     <row r="7" spans="1:26">
       <c r="A7" t="s">
-        <v>94</v>
+        <v>113</v>
       </c>
       <c r="B7" t="s">
-        <v>82</v>
+        <v>114</v>
       </c>
       <c r="C7">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="8" spans="1:26">
+      <c r="A8" t="s">
+        <v>115</v>
+      </c>
+      <c r="B8" t="s">
+        <v>91</v>
+      </c>
+      <c r="C8">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="9" spans="1:26">
+      <c r="A9" t="s">
+        <v>116</v>
+      </c>
+      <c r="B9" t="s">
+        <v>93</v>
+      </c>
+      <c r="C9">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="10" spans="1:26">
+      <c r="A10" t="s">
+        <v>117</v>
+      </c>
+      <c r="B10" t="s">
+        <v>95</v>
+      </c>
+      <c r="C10">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="11" spans="1:26">
+      <c r="A11" t="s">
+        <v>118</v>
+      </c>
+      <c r="B11" t="s">
+        <v>119</v>
+      </c>
+      <c r="C11">
         <v>1</v>
       </c>
     </row>
@@ -1489,7 +1710,7 @@
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
   </sheetPr>
-  <dimension ref="A1:Z8"/>
+  <dimension ref="A1:Z9"/>
   <sheetFormatPr defaultRowHeight="14.4" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col min="1" max="1" width="28" customWidth="true" style="0"/>
@@ -1501,19 +1722,19 @@
   <sheetData>
     <row r="1" spans="1:26">
       <c r="A1" s="2" t="s">
-        <v>95</v>
+        <v>120</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>96</v>
+        <v>121</v>
       </c>
       <c r="C1" s="2" t="s">
-        <v>97</v>
+        <v>122</v>
       </c>
       <c r="D1" s="2" t="s">
-        <v>98</v>
+        <v>123</v>
       </c>
       <c r="E1" s="2" t="s">
-        <v>99</v>
+        <v>124</v>
       </c>
       <c r="F1" s="2"/>
       <c r="G1" s="2"/>
@@ -1539,19 +1760,19 @@
     </row>
     <row r="2" spans="1:26">
       <c r="A2" s="1" t="s">
-        <v>100</v>
+        <v>125</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>101</v>
+        <v>126</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>11</v>
+        <v>18</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>102</v>
+        <v>127</v>
       </c>
       <c r="E2" s="1" t="s">
-        <v>19</v>
+        <v>26</v>
       </c>
       <c r="F2" s="1"/>
       <c r="G2" s="1"/>
@@ -1577,104 +1798,121 @@
     </row>
     <row r="3" spans="1:26">
       <c r="A3" t="s">
-        <v>103</v>
+        <v>128</v>
       </c>
       <c r="B3" t="s">
-        <v>104</v>
+        <v>129</v>
       </c>
       <c r="C3">
         <v>1</v>
       </c>
       <c r="D3" t="s">
-        <v>89</v>
+        <v>108</v>
       </c>
       <c r="E3" t="s">
-        <v>74</v>
+        <v>81</v>
       </c>
     </row>
     <row r="4" spans="1:26">
       <c r="A4" t="s">
-        <v>105</v>
+        <v>128</v>
       </c>
       <c r="B4" t="s">
-        <v>106</v>
+        <v>129</v>
       </c>
       <c r="C4">
         <v>1</v>
       </c>
       <c r="D4" t="s">
-        <v>89</v>
+        <v>108</v>
       </c>
       <c r="E4" t="s">
-        <v>74</v>
+        <v>83</v>
       </c>
     </row>
     <row r="5" spans="1:26">
       <c r="A5" t="s">
-        <v>105</v>
+        <v>130</v>
       </c>
       <c r="B5" t="s">
-        <v>106</v>
+        <v>131</v>
       </c>
       <c r="C5">
         <v>1</v>
       </c>
       <c r="D5" t="s">
-        <v>89</v>
+        <v>110</v>
       </c>
       <c r="E5" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
     </row>
     <row r="6" spans="1:26">
       <c r="A6" t="s">
-        <v>107</v>
+        <v>132</v>
       </c>
       <c r="B6" t="s">
-        <v>108</v>
+        <v>133</v>
       </c>
       <c r="C6">
         <v>1</v>
       </c>
       <c r="D6" t="s">
-        <v>91</v>
+        <v>106</v>
       </c>
       <c r="E6" t="s">
-        <v>76</v>
+        <v>87</v>
       </c>
     </row>
     <row r="7" spans="1:26">
       <c r="A7" t="s">
-        <v>109</v>
+        <v>134</v>
       </c>
       <c r="B7" t="s">
-        <v>110</v>
+        <v>135</v>
       </c>
       <c r="C7">
         <v>1</v>
       </c>
       <c r="D7" t="s">
-        <v>92</v>
+        <v>116</v>
       </c>
       <c r="E7" t="s">
-        <v>78</v>
+        <v>93</v>
       </c>
     </row>
     <row r="8" spans="1:26">
       <c r="A8" t="s">
-        <v>111</v>
+        <v>136</v>
       </c>
       <c r="B8" t="s">
-        <v>112</v>
+        <v>137</v>
       </c>
       <c r="C8">
         <v>1</v>
       </c>
       <c r="D8" t="s">
-        <v>93</v>
+        <v>118</v>
       </c>
       <c r="E8" t="s">
-        <v>80</v>
+        <v>89</v>
+      </c>
+    </row>
+    <row r="9" spans="1:26">
+      <c r="A9" t="s">
+        <v>136</v>
+      </c>
+      <c r="B9" t="s">
+        <v>137</v>
+      </c>
+      <c r="C9">
+        <v>1</v>
+      </c>
+      <c r="D9" t="s">
+        <v>118</v>
+      </c>
+      <c r="E9" t="s">
+        <v>99</v>
       </c>
     </row>
   </sheetData>

</xml_diff>